<commit_message>
Chaos upgrades (from db.xlsx)
- DATA.chaos: 10 modifiers (provisional names) with max Lv and points per Lv, reward table every 5 points up to 60
- Stage select: cleared entries show their chaos points and a 設定 button opening a panel to raise/lower each modifier; saved per mode/stage in META.chaos
- Run effects (CHAOS): enemy level speed, +Lv per boss kill, starting Lv, spawn rate/cap, enemy attack area (warnings, hitCircle/hitLine, projectiles, hazards, direct checks), enemy attack frequency (boss AI cooldowns, archer shots), fewer item drops (not chests), longer debuffs, bosses always enraged, twin bosses (a random other-stage boss; progress only when both fall)
- Rewards enter stats as source 'カオス強化' for that run (roll cap, equipment Lv cap, equipment/chest quality, gold)
- Design doc 9 documents the modifiers

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/claudedocs/db.xlsx
+++ b/claudedocs/db.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Black\Desktop\pixel_survivors\pixel_survivors_opus5.5test\claudedocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{897A5F9F-63DA-495F-A521-7F999B482F49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38848A7F-ADCC-4C4D-89BF-E3B7C0ED2529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1335" yWindow="2175" windowWidth="27390" windowHeight="14400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10950" yWindow="3525" windowWidth="27390" windowHeight="14400" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ステータス" sheetId="2" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="バフデバフ" sheetId="3" r:id="rId3"/>
     <sheet name="クラス一覧" sheetId="1" r:id="rId4"/>
     <sheet name="クラスレベル" sheetId="5" r:id="rId5"/>
+    <sheet name="カオス強化" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="192">
   <si>
     <t>クラス</t>
     <phoneticPr fontId="1"/>
@@ -933,6 +934,567 @@
   </si>
   <si>
     <t>武器枠+1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>カオス名</t>
+    <rPh sb="3" eb="4">
+      <t>メイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最大レベル</t>
+    <rPh sb="0" eb="2">
+      <t>サイダイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>レベルの上昇速度+20%</t>
+    <rPh sb="4" eb="6">
+      <t>ジョウショウ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ソクド</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ボス討伐時にレベル１上昇</t>
+    <rPh sb="2" eb="4">
+      <t>トウバツ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>ジ</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>ジョウショウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>敵の出現率+5%</t>
+    <rPh sb="0" eb="1">
+      <t>テキ</t>
+    </rPh>
+    <rPh sb="2" eb="5">
+      <t>シュツゲンリツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ボスは同時に２種類出現する</t>
+    <rPh sb="3" eb="5">
+      <t>ドウジ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>シュルイ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>シュツゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ボスは常に激怒する</t>
+    <rPh sb="3" eb="4">
+      <t>ツネ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ゲキド</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ポイント</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>敵の攻撃頻度+10%</t>
+    <rPh sb="0" eb="1">
+      <t>テキ</t>
+    </rPh>
+    <rPh sb="2" eb="6">
+      <t>コウゲキヒンド</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>敵の攻撃範囲+10%</t>
+    <rPh sb="0" eb="1">
+      <t>テキ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>コウゲキ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ハンイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>初期レベル+1</t>
+    <rPh sb="0" eb="2">
+      <t>ショキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備ロール上限+5%</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備ロール上限+10%</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>報酬１</t>
+    <rPh sb="0" eb="2">
+      <t>ホウシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>報酬2</t>
+    <rPh sb="0" eb="2">
+      <t>ホウシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>報酬3</t>
+    <rPh sb="0" eb="2">
+      <t>ホウシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備ロール上限+15%</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備ロール上限+20%</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備ロール上限+25%</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備ロール上限+30%</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備ロール上限+35%</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備ロール上限+40%</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備ロール上限+45%</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備ロール上限+50%</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備Lv上限+2</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備Lv上限+1</t>
+    <rPh sb="0" eb="2">
+      <t>ソウビ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ジョウゲン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>報酬4</t>
+    <rPh sb="0" eb="2">
+      <t>ホウシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+5%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+10%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+15%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+20%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+25%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+30%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+35%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+40%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+45%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+50%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+10%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+20%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+30%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+40%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+50%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+60%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+70%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+80%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+90%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+100%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>報酬5</t>
+    <rPh sb="0" eb="2">
+      <t>ホウシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+20%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+40%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+60%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+80%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+100%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+120%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+140%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+160%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+180%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+200%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>アイテムの出現率-10%</t>
+    <rPh sb="5" eb="8">
+      <t>シュツゲンリツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>デバフの効果時間+10%</t>
+    <rPh sb="4" eb="8">
+      <t>コウカジカン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+120%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>装備品質+150%</t>
+    <rPh sb="0" eb="4">
+      <t>ソウビヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+75%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宝箱品質+100%</t>
+    <rPh sb="0" eb="2">
+      <t>タカラバコ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒンシツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+250%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>獲得ゴールド+300%</t>
+    <rPh sb="0" eb="2">
+      <t>カクトク</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1021,7 +1583,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1046,6 +1608,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -2703,4 +3268,402 @@
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09DF0200-B449-4DD1-9AB3-A7EB3E24320C}">
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="1" max="1" width="22.5" customWidth="1"/>
+    <col min="2" max="3" width="19.875" style="10" customWidth="1"/>
+    <col min="4" max="4" width="19.875" customWidth="1"/>
+    <col min="5" max="5" width="19.625" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="8" width="8.375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="2" customFormat="1" ht="35.25" customHeight="1">
+      <c r="A1" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="B2" s="10">
+        <v>5</v>
+      </c>
+      <c r="C2" s="10">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="B3" s="10">
+        <v>5</v>
+      </c>
+      <c r="C3" s="10">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="B4" s="10">
+        <v>4</v>
+      </c>
+      <c r="C4" s="10">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="B5" s="10">
+        <v>5</v>
+      </c>
+      <c r="C5" s="10">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="B6" s="10">
+        <v>5</v>
+      </c>
+      <c r="C6" s="10">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="B7" s="10">
+        <v>3</v>
+      </c>
+      <c r="C7" s="10">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="B8" s="10">
+        <v>5</v>
+      </c>
+      <c r="C8" s="10">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="B9" s="10">
+        <v>5</v>
+      </c>
+      <c r="C9" s="10">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="B10" s="10">
+        <v>1</v>
+      </c>
+      <c r="C10" s="10">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="B11" s="10">
+        <v>1</v>
+      </c>
+      <c r="C11" s="10">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="24">
+      <c r="A13" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="10">
+        <v>5</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="E14" t="s">
+        <v>153</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="10">
+        <v>10</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="E15" t="s">
+        <v>154</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="10">
+        <v>15</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="E16" t="s">
+        <v>155</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="10">
+        <v>20</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="E17" t="s">
+        <v>156</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="10">
+        <v>25</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="E18" t="s">
+        <v>157</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="10">
+        <v>30</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="E19" t="s">
+        <v>158</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="10">
+        <v>35</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="E20" t="s">
+        <v>159</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="10">
+        <v>40</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="E21" t="s">
+        <v>160</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="10">
+        <v>45</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="E22" t="s">
+        <v>161</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="10">
+        <v>50</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="E23" t="s">
+        <v>162</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="10">
+        <v>55</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="E24" t="s">
+        <v>188</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="10">
+        <v>60</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="E25" t="s">
+        <v>189</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="10"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>